<commit_message>
Reset Excel Table for FORKLIFT-01
</commit_message>
<xml_diff>
--- a/FM-MN-07_FORKLIFT-01.xlsx
+++ b/FM-MN-07_FORKLIFT-01.xlsx
@@ -1735,17 +1735,9 @@
           <t>ตรวจเช็คระบบน้ำหม้อน้ำให้อยู่ในระดับ Hight</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="9" t="inlineStr"/>
       <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E6" s="9" t="inlineStr"/>
       <c r="F6" s="9" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
       <c r="H6" s="9" t="inlineStr"/>
@@ -1784,11 +1776,7 @@
           <t>ตรวจเช็คน้ำมันเครื่องยนต์ต้องอยู่ไม่เกินขีดที่3ของตัวเช็ค</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="9" t="inlineStr"/>
       <c r="D7" s="9" t="inlineStr"/>
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="9" t="inlineStr"/>
@@ -1829,11 +1817,7 @@
           <t>ตรวจเช็คไส้กรองและเป่าลมทำความสะอาด</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C8" s="9" t="inlineStr"/>
       <c r="D8" s="9" t="inlineStr"/>
       <c r="E8" s="9" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr"/>
@@ -1874,17 +1858,9 @@
           <t>ตรวจเช็คการรั่วซึมของน้ำมันไฮดรอริก</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="9" t="inlineStr"/>
       <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E9" s="9" t="inlineStr"/>
       <c r="F9" s="9" t="inlineStr"/>
       <c r="G9" s="9" t="inlineStr"/>
       <c r="H9" s="9" t="inlineStr"/>
@@ -1923,17 +1899,9 @@
           <t>ตรวจเช็คระบบเบรคและน้ำมันเบรค</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C10" s="9" t="inlineStr"/>
       <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E10" s="9" t="inlineStr"/>
       <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr"/>
       <c r="H10" s="9" t="inlineStr"/>
@@ -1972,17 +1940,9 @@
           <t>ตรวจเช็คไฟส่องสว่างและไฟเลี้ยว</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C11" s="9" t="inlineStr"/>
       <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E11" s="9" t="inlineStr"/>
       <c r="F11" s="9" t="inlineStr"/>
       <c r="G11" s="9" t="inlineStr"/>
       <c r="H11" s="9" t="inlineStr"/>
@@ -2056,17 +2016,9 @@
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="7" t="n"/>
       <c r="B13" s="6" t="n"/>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>คะนอง บัวจันทร์</t>
-        </is>
-      </c>
+      <c r="C13" s="43" t="inlineStr"/>
       <c r="D13" s="40" t="inlineStr"/>
-      <c r="E13" s="43" t="inlineStr">
-        <is>
-          <t>คะนอง บัวจันทร์</t>
-        </is>
-      </c>
+      <c r="E13" s="43" t="inlineStr"/>
       <c r="F13" s="40" t="inlineStr"/>
       <c r="G13" s="40" t="inlineStr"/>
       <c r="H13" s="40" t="inlineStr"/>
@@ -2206,11 +2158,7 @@
       </c>
     </row>
     <row r="18" ht="224.25" customHeight="1">
-      <c r="B18" s="41" t="inlineStr">
-        <is>
-          <t>[วันที่ 1]: หน้าปัดมองไม่ชัด,  [วันที่ 3]: หน้าปัดมองไม่ชัด</t>
-        </is>
-      </c>
+      <c r="B18" s="41" t="inlineStr"/>
     </row>
     <row r="19" ht="23.25" customHeight="1"/>
     <row r="20" ht="23.25" customHeight="1">

</xml_diff>

<commit_message>
Direct Write Excel for FORKLIFT-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_FORKLIFT-01.xlsx
+++ b/FM-MN-07_FORKLIFT-01.xlsx
@@ -1740,7 +1740,11 @@
       <c r="E6" s="9" t="inlineStr"/>
       <c r="F6" s="9" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
@@ -1781,7 +1785,11 @@
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="9" t="inlineStr"/>
       <c r="G7" s="9" t="inlineStr"/>
-      <c r="H7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="9" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
@@ -1822,7 +1830,11 @@
       <c r="E8" s="9" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="9" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
@@ -1863,7 +1875,11 @@
       <c r="E9" s="9" t="inlineStr"/>
       <c r="F9" s="9" t="inlineStr"/>
       <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
@@ -1904,7 +1920,11 @@
       <c r="E10" s="9" t="inlineStr"/>
       <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="9" t="inlineStr"/>
       <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
@@ -1945,7 +1965,11 @@
       <c r="E11" s="9" t="inlineStr"/>
       <c r="F11" s="9" t="inlineStr"/>
       <c r="G11" s="9" t="inlineStr"/>
-      <c r="H11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
@@ -1986,7 +2010,11 @@
       <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="9" t="inlineStr"/>
       <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
@@ -2021,7 +2049,11 @@
       <c r="E13" s="43" t="inlineStr"/>
       <c r="F13" s="40" t="inlineStr"/>
       <c r="G13" s="40" t="inlineStr"/>
-      <c r="H13" s="40" t="inlineStr"/>
+      <c r="H13" s="43" t="inlineStr">
+        <is>
+          <t>คะนอง บัวจันทร์</t>
+        </is>
+      </c>
       <c r="I13" s="40" t="inlineStr"/>
       <c r="J13" s="40" t="inlineStr"/>
       <c r="K13" s="40" t="inlineStr"/>
@@ -2158,7 +2190,11 @@
       </c>
     </row>
     <row r="18" ht="224.25" customHeight="1">
-      <c r="B18" s="41" t="inlineStr"/>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>[วันที่ 6]: ข้อ 2: หน้าปัดมองไม่ชัด, ข้อ 5: หน้าปัดมองไม่ชัด</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="23.25" customHeight="1"/>
     <row r="20" ht="23.25" customHeight="1">

</xml_diff>

<commit_message>
Safe Direct Write Excel for FORKLIFT-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_FORKLIFT-01.xlsx
+++ b/FM-MN-07_FORKLIFT-01.xlsx
@@ -1745,7 +1745,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr"/>
@@ -1790,7 +1794,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr"/>
@@ -1835,7 +1843,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
       <c r="L8" s="9" t="inlineStr"/>
@@ -1880,7 +1892,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr"/>
@@ -1925,7 +1941,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="9" t="inlineStr"/>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr"/>
@@ -1970,7 +1990,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
@@ -2015,7 +2039,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr"/>
@@ -2054,7 +2082,11 @@
           <t>คะนอง บัวจันทร์</t>
         </is>
       </c>
-      <c r="I13" s="40" t="inlineStr"/>
+      <c r="I13" s="43" t="inlineStr">
+        <is>
+          <t>คะนอง บัวจันทร์</t>
+        </is>
+      </c>
       <c r="J13" s="40" t="inlineStr"/>
       <c r="K13" s="40" t="inlineStr"/>
       <c r="L13" s="40" t="inlineStr"/>
@@ -2192,7 +2224,7 @@
     <row r="18" ht="224.25" customHeight="1">
       <c r="B18" s="41" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 2: หน้าปัดมองไม่ชัด, ข้อ 5: หน้าปัดมองไม่ชัด</t>
+          <t>[วันที่ 6]: ข้อ 2: หน้าปัดมองไม่ชัด, ข้อ 5: หน้าปัดมองไม่ชัด,  [วันที่ 7]: ข้อ 2: หน้าปัดมองไม่ชัด</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for FORKLIFT-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_FORKLIFT-01.xlsx
+++ b/FM-MN-07_FORKLIFT-01.xlsx
@@ -1750,7 +1750,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr"/>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="9" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr"/>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="9" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr"/>
       <c r="M7" s="9" t="inlineStr"/>
@@ -1848,7 +1856,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="9" t="inlineStr"/>
       <c r="L8" s="9" t="inlineStr"/>
       <c r="M8" s="9" t="inlineStr"/>
@@ -1897,7 +1909,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr"/>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="9" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr"/>
       <c r="M9" s="9" t="inlineStr"/>
@@ -1946,7 +1962,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="9" t="inlineStr"/>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr"/>
@@ -1995,7 +2015,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="9" t="inlineStr"/>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="9" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
       <c r="M11" s="9" t="inlineStr"/>
@@ -2044,7 +2068,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="9" t="inlineStr"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr"/>
@@ -2087,7 +2115,11 @@
           <t>คะนอง บัวจันทร์</t>
         </is>
       </c>
-      <c r="J13" s="40" t="inlineStr"/>
+      <c r="J13" s="43" t="inlineStr">
+        <is>
+          <t>คะนอง บัวจันทร์</t>
+        </is>
+      </c>
       <c r="K13" s="40" t="inlineStr"/>
       <c r="L13" s="40" t="inlineStr"/>
       <c r="M13" s="40" t="inlineStr"/>
@@ -2224,7 +2256,7 @@
     <row r="18" ht="224.25" customHeight="1">
       <c r="B18" s="41" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 2: หน้าปัดมองไม่ชัด, ข้อ 5: หน้าปัดมองไม่ชัด,  [วันที่ 7]: ข้อ 2: หน้าปัดมองไม่ชัด,  [วันที่ 7]: ข้อ 5: หน้าปัดมองไม่ชัด</t>
+          <t>[วันที่ 6]: ข้อ 2: หน้าปัดมองไม่ชัด, ข้อ 5: หน้าปัดมองไม่ชัด,  [วันที่ 7]: ข้อ 2: หน้าปัดมองไม่ชัด,  [วันที่ 7]: ข้อ 5: หน้าปัดมองไม่ชัด,  [วันที่ 8]: ข้อ 2: หน้าปัดมองไม่ชัด, ข้อ 5: หน้าปัดมองไม่ชัด</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Safe Direct Write Excel for FORKLIFT-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_FORKLIFT-01.xlsx
+++ b/FM-MN-07_FORKLIFT-01.xlsx
@@ -1756,7 +1756,11 @@
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="9" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="9" t="inlineStr"/>
       <c r="N6" s="9" t="inlineStr"/>
       <c r="O6" s="9" t="inlineStr"/>
@@ -1809,7 +1813,11 @@
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="9" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="9" t="inlineStr"/>
       <c r="N7" s="9" t="inlineStr"/>
       <c r="O7" s="9" t="inlineStr"/>
@@ -1862,7 +1870,11 @@
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="9" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="9" t="inlineStr"/>
       <c r="N8" s="9" t="inlineStr"/>
       <c r="O8" s="9" t="inlineStr"/>
@@ -1915,7 +1927,11 @@
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr"/>
-      <c r="L9" s="9" t="inlineStr"/>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="9" t="inlineStr"/>
       <c r="N9" s="9" t="inlineStr"/>
       <c r="O9" s="9" t="inlineStr"/>
@@ -1968,7 +1984,11 @@
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="9" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="9" t="inlineStr"/>
       <c r="N10" s="9" t="inlineStr"/>
       <c r="O10" s="9" t="inlineStr"/>
@@ -2021,7 +2041,11 @@
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="9" t="inlineStr"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="9" t="inlineStr"/>
       <c r="N11" s="9" t="inlineStr"/>
       <c r="O11" s="9" t="inlineStr"/>
@@ -2074,7 +2098,11 @@
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr"/>
-      <c r="L12" s="9" t="inlineStr"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="9" t="inlineStr"/>
       <c r="N12" s="9" t="inlineStr"/>
       <c r="O12" s="9" t="inlineStr"/>
@@ -2121,7 +2149,11 @@
         </is>
       </c>
       <c r="K13" s="40" t="inlineStr"/>
-      <c r="L13" s="40" t="inlineStr"/>
+      <c r="L13" s="43" t="inlineStr">
+        <is>
+          <t>คะนอง บัวจันทร์</t>
+        </is>
+      </c>
       <c r="M13" s="40" t="inlineStr"/>
       <c r="N13" s="40" t="inlineStr"/>
       <c r="O13" s="40" t="inlineStr"/>

</xml_diff>